<commit_message>
Sprint 5 completed - Production Dashboard and Deployment
</commit_message>
<xml_diff>
--- a/n100/output/peer_comparison.xlsx
+++ b/n100/output/peer_comparison.xlsx
@@ -678,12 +678,14 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>-14556</v>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -702,12 +704,14 @@
           <t>25.0%</t>
         </is>
       </c>
-      <c r="R2" t="n">
-        <v>35.1</v>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>75.0%</t>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -775,12 +779,14 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>35669</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -799,8 +805,10 @@
           <t>100.0%</t>
         </is>
       </c>
-      <c r="R3" t="n">
-        <v>15.42</v>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
@@ -872,12 +880,14 @@
           <t>75.0%</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>12547</v>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>75.0%</t>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N4" t="n">
@@ -896,12 +906,14 @@
           <t>75.0%</t>
         </is>
       </c>
-      <c r="R4" t="n">
-        <v>55.18</v>
-      </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -969,8 +981,10 @@
           <t>25.0%</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>-17468</v>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
@@ -993,12 +1007,14 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="R5" t="n">
-        <v>15.9</v>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="T5" t="n">
@@ -1066,12 +1082,14 @@
           <t>100.0%</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>6766</v>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N6" t="n">
@@ -1090,12 +1108,14 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="R6" t="n">
-        <v>19.34</v>
-      </c>
-      <c r="S6" s="4" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -1163,8 +1183,10 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>6766</v>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
@@ -1187,8 +1209,10 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>19.34</v>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="S7" s="6" t="inlineStr">
         <is>
@@ -3108,12 +3132,14 @@
           <t>33.3%</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>-7559</v>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>33.3%</t>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -3132,12 +3158,14 @@
           <t>66.7%</t>
         </is>
       </c>
-      <c r="R2" t="n">
-        <v>55.18</v>
-      </c>
-      <c r="S2" s="4" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -3205,12 +3233,14 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>13296</v>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>66.7%</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -3229,8 +3259,10 @@
           <t>100.0%</t>
         </is>
       </c>
-      <c r="R3" t="n">
-        <v>53.42</v>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
@@ -3302,8 +3334,10 @@
           <t>66.7%</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>-29445</v>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
@@ -3407,12 +3441,14 @@
           <t>100.0%</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>18156</v>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -3431,12 +3467,14 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="R5" t="n">
-        <v>90.37</v>
-      </c>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="T5" t="n">
@@ -3506,8 +3544,10 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="L6" s="6" t="n">
-        <v>2868.5</v>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
@@ -3530,8 +3570,10 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="R6" s="6" t="n">
-        <v>55.18</v>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
         <is>

</xml_diff>